<commit_message>
More 1 user test
</commit_message>
<xml_diff>
--- a/UserTests/Results/UserTestResultsWave2.xlsx
+++ b/UserTests/Results/UserTestResultsWave2.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <x:si>
     <x:t xml:space="preserve">ID</x:t>
   </x:si>
@@ -93,6 +93,12 @@
     <x:t xml:space="preserve">12</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">13</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">14</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">I think that I would like to use this system frequently.</x:t>
   </x:si>
   <x:si>
@@ -124,6 +130,10 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">What did you like most and less about the game.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Do you have any suggestions, comments, or thoughts about your experience with the personalized XR session?
+</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Other Suggestions</x:t>
@@ -222,6 +232,12 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">The button that you need to press sometimes doesnt work properly. It works better when you press with one finger than with the whole hand open.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Gosto bastanto do jogo em si, está muito bem concebido. Tanto acerca do cenário como dos mini-jogos. Além de ser útil para a reabiliação tambem é divertido :D</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Diria que podia haver um acréscimo de pontos caso a sequência fosse cada vez maior.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -318,9 +334,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AH9" insertRow="1" totalsRowShown="0">
-  <x:autoFilter ref="A1:AH9"/>
-  <x:tableColumns count="34">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK10" insertRow="1" totalsRowShown="0">
+  <x:autoFilter ref="A1:AK10"/>
+  <x:tableColumns count="37">
     <x:tableColumn id="1" uniqueName="1" name="ID" dataDxfId="0"/>
     <x:tableColumn id="2" uniqueName="2" name="Start time" dataDxfId="3"/>
     <x:tableColumn id="3" uniqueName="3" name="Completion time" dataDxfId="3"/>
@@ -343,18 +359,21 @@
     <x:tableColumn id="20" uniqueName="20" name="10" dataDxfId="0"/>
     <x:tableColumn id="21" uniqueName="21" name="11" dataDxfId="0"/>
     <x:tableColumn id="22" uniqueName="22" name="12" dataDxfId="0"/>
-    <x:tableColumn id="23" uniqueName="23" name="I think that I would like to use this system frequently." dataDxfId="0"/>
-    <x:tableColumn id="24" uniqueName="24" name="I found the system unnecessarily complex." dataDxfId="0"/>
-    <x:tableColumn id="25" uniqueName="25" name="I thought the system was easy to use." dataDxfId="0"/>
-    <x:tableColumn id="26" uniqueName="26" name="I think that I would need the support of a technical person to be able to use ." dataDxfId="0"/>
-    <x:tableColumn id="27" uniqueName="27" name="I found the various functions in the system were well integrated." dataDxfId="0"/>
-    <x:tableColumn id="28" uniqueName="28" name="I thought there was too much inconsistency in this system." dataDxfId="0"/>
-    <x:tableColumn id="29" uniqueName="29" name="I imagine that most people would learn to use this product very quickly." dataDxfId="0"/>
-    <x:tableColumn id="30" uniqueName="30" name="I found the product very awkward to use." dataDxfId="0"/>
-    <x:tableColumn id="31" uniqueName="31" name="I felt very confident using the product" dataDxfId="0"/>
-    <x:tableColumn id="32" uniqueName="32" name="I needed to learn a lot of things before I could get going with this product." dataDxfId="0"/>
-    <x:tableColumn id="33" uniqueName="33" name="What did you like most and less about the game." dataDxfId="0"/>
-    <x:tableColumn id="34" uniqueName="34" name="Other Suggestions" dataDxfId="0"/>
+    <x:tableColumn id="23" uniqueName="23" name="13" dataDxfId="0"/>
+    <x:tableColumn id="24" uniqueName="24" name="14" dataDxfId="0"/>
+    <x:tableColumn id="25" uniqueName="25" name="I think that I would like to use this system frequently." dataDxfId="0"/>
+    <x:tableColumn id="26" uniqueName="26" name="I found the system unnecessarily complex." dataDxfId="0"/>
+    <x:tableColumn id="27" uniqueName="27" name="I thought the system was easy to use." dataDxfId="0"/>
+    <x:tableColumn id="28" uniqueName="28" name="I think that I would need the support of a technical person to be able to use ." dataDxfId="0"/>
+    <x:tableColumn id="29" uniqueName="29" name="I found the various functions in the system were well integrated." dataDxfId="0"/>
+    <x:tableColumn id="30" uniqueName="30" name="I thought there was too much inconsistency in this system." dataDxfId="0"/>
+    <x:tableColumn id="31" uniqueName="31" name="I imagine that most people would learn to use this product very quickly." dataDxfId="0"/>
+    <x:tableColumn id="32" uniqueName="32" name="I found the product very awkward to use." dataDxfId="0"/>
+    <x:tableColumn id="33" uniqueName="33" name="I felt very confident using the product" dataDxfId="0"/>
+    <x:tableColumn id="34" uniqueName="34" name="I needed to learn a lot of things before I could get going with this product." dataDxfId="0"/>
+    <x:tableColumn id="35" uniqueName="35" name="What did you like most and less about the game." dataDxfId="0"/>
+    <x:tableColumn id="36" uniqueName="36" name="Do you have any suggestions, comments, or thoughts about your experience with the personalized XR session?&#10;" dataDxfId="0"/>
+    <x:tableColumn id="37" uniqueName="37" name="Other Suggestions" dataDxfId="0"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -694,6 +713,9 @@
     <x:col min="32" max="32" width="20" hidden="0" bestFit="1" customWidth="1"/>
     <x:col min="33" max="33" width="20" hidden="0" bestFit="1" customWidth="1"/>
     <x:col min="34" max="34" width="20" hidden="0" bestFit="1" customWidth="1"/>
+    <x:col min="35" max="35" width="20" hidden="0" bestFit="1" customWidth="1"/>
+    <x:col min="36" max="36" width="20" hidden="0" bestFit="1" customWidth="1"/>
+    <x:col min="37" max="37" width="20" hidden="0" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" hidden="0">
@@ -763,10 +785,10 @@
       <x:c r="V1" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="W1" s="10" t="s">
+      <x:c r="W1" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="X1" s="10" t="s">
+      <x:c r="X1" s="7" t="s">
         <x:v>23</x:v>
       </x:c>
       <x:c r="Y1" s="10" t="s">
@@ -798,6 +820,15 @@
       </x:c>
       <x:c r="AH1" s="10" t="s">
         <x:v>33</x:v>
+      </x:c>
+      <x:c r="AI1" s="10" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="AJ1" s="10" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="AK1" s="10" t="s">
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="2" hidden="0">
@@ -811,93 +842,96 @@
         <x:v>46090.4489236111</x:v>
       </x:c>
       <x:c r="D2" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E2" s="10" t="s"/>
       <x:c r="F2" s="2"/>
       <x:c r="G2" s="7" t="s">
-        <x:v>35</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="H2" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="I2" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="J2" s="10" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="K2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="L2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M2" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="N2" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="O2" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="P2" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Q2" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="R2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="S2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="T2" s="10" t="s">
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="U2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="V2" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="W2" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="X2" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="W2" s="10" t="s"/>
+      <x:c r="X2" s="10" t="s"/>
       <x:c r="Y2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="Z2" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AA2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AB2" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AC2" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AD2" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AE2" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AF2" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AG2" s="10" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AH2" s="10" t="s">
-        <x:v>44</x:v>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI2" s="10" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="AJ2" s="10" t="s"/>
+      <x:c r="AK2" s="10" t="s">
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="3" hidden="0">
@@ -911,93 +945,96 @@
         <x:v>46090.4594212963</x:v>
       </x:c>
       <x:c r="D3" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E3" s="10" t="s"/>
       <x:c r="F3" s="2"/>
       <x:c r="G3" s="7" t="s">
-        <x:v>45</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="H3" s="10" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I3" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="J3" s="10" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="K3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="L3" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="N3" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="O3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="P3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Q3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="R3" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="S3" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="T3" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="U3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="V3" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="W3" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="X3" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W3" s="10" t="s"/>
+      <x:c r="X3" s="10" t="s"/>
       <x:c r="Y3" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="Z3" s="10" t="s">
-        <x:v>41</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AA3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AB3" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="AC3" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AD3" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AE3" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AF3" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AG3" s="10" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AH3" s="10" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AI3" s="10" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="AJ3" s="10" t="s"/>
+      <x:c r="AK3" s="10" t="s">
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="4" hidden="0">
@@ -1011,89 +1048,92 @@
         <x:v>46090.6165393519</x:v>
       </x:c>
       <x:c r="D4" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E4" s="10" t="s"/>
       <x:c r="F4" s="2"/>
       <x:c r="G4" s="7" t="s">
-        <x:v>50</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="H4" s="10" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I4" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="J4" s="10" t="s">
-        <x:v>51</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="K4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="L4" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="N4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="O4" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="P4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Q4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="R4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="S4" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="T4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="U4" s="10" t="s"/>
       <x:c r="V4" s="10" t="s"/>
-      <x:c r="W4" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="X4" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
+      <x:c r="W4" s="10" t="s"/>
+      <x:c r="X4" s="10" t="s"/>
       <x:c r="Y4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="Z4" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AA4" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AB4" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AC4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AD4" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AE4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AF4" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AG4" s="10" t="s">
-        <x:v>52</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AH4" s="10" t="s">
-        <x:v>53</x:v>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI4" s="10" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="AJ4" s="10" t="s"/>
+      <x:c r="AK4" s="10" t="s">
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="5" hidden="0">
@@ -1107,93 +1147,96 @@
         <x:v>46090.7401157407</x:v>
       </x:c>
       <x:c r="D5" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s"/>
       <x:c r="F5" s="2"/>
       <x:c r="G5" s="7" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="H5" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I5" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J5" s="10" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="H5" s="10" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="I5" s="10" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="J5" s="10" t="s">
-        <x:v>51</x:v>
-      </x:c>
       <x:c r="K5" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="L5" s="10" t="s">
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="M5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="N5" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="O5" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="P5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Q5" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="R5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="S5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="T5" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="U5" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="V5" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="W5" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="X5" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W5" s="10" t="s"/>
+      <x:c r="X5" s="10" t="s"/>
       <x:c r="Y5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Z5" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AA5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AB5" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AC5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AD5" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AE5" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AF5" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AG5" s="10" t="s">
-        <x:v>55</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AH5" s="10" t="s">
-        <x:v>56</x:v>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI5" s="10" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="AJ5" s="10" t="s"/>
+      <x:c r="AK5" s="10" t="s">
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="6" hidden="0">
@@ -1207,92 +1250,95 @@
         <x:v>46090.7478240741</x:v>
       </x:c>
       <x:c r="D6" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E6" s="10" t="s"/>
       <x:c r="F6" s="2"/>
       <x:c r="G6" s="7" t="s">
-        <x:v>57</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H6" s="10" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I6" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="J6" s="10" t="s">
-        <x:v>51</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="K6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="L6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M6" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="N6" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="O6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="P6" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Q6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="R6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="S6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="T6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="U6" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="V6" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="W6" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="X6" s="10" t="s">
-        <x:v>47</x:v>
-      </x:c>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W6" s="10" t="s"/>
+      <x:c r="X6" s="10" t="s"/>
       <x:c r="Y6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="Z6" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AA6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AB6" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AC6" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AD6" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AE6" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AF6" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AG6" s="10" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="AH6" s="10" t="s"/>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH6" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI6" s="10" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="AJ6" s="10" t="s"/>
+      <x:c r="AK6" s="10" t="s"/>
     </x:row>
     <x:row r="7" hidden="0">
       <x:c r="A7">
@@ -1305,92 +1351,95 @@
         <x:v>46091.697337963</x:v>
       </x:c>
       <x:c r="D7" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E7" s="10" t="s"/>
       <x:c r="F7" s="2"/>
       <x:c r="G7" s="7" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="H7" s="10" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="I7" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J7" s="10" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="H7" s="10" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="I7" s="10" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="J7" s="10" t="s">
-        <x:v>51</x:v>
-      </x:c>
       <x:c r="K7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="L7" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="M7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="N7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="O7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="P7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="Q7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="R7" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="S7" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="T7" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="U7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="V7" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="W7" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="X7" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W7" s="10" t="s"/>
+      <x:c r="X7" s="10" t="s"/>
       <x:c r="Y7" s="10" t="s">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="Z7" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AA7" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="AB7" s="10" t="s">
         <x:v>42</x:v>
       </x:c>
       <x:c r="AC7" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AD7" s="10" t="s">
-        <x:v>41</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AE7" s="10" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="AF7" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="AG7" s="10" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="AH7" s="10" t="s"/>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AH7" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI7" s="10" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="AJ7" s="10" t="s"/>
+      <x:c r="AK7" s="10" t="s"/>
     </x:row>
     <x:row r="8" hidden="0">
       <x:c r="A8">
@@ -1403,92 +1452,95 @@
         <x:v>46091.7214467593</x:v>
       </x:c>
       <x:c r="D8" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E8" s="10" t="s"/>
       <x:c r="F8" s="2"/>
       <x:c r="G8" s="7" t="s">
-        <x:v>60</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H8" s="10" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I8" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="J8" s="10" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="K8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="L8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="N8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="O8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="P8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="Q8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="R8" s="10" t="s">
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="S8" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="T8" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="U8" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="V8" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="W8" s="10" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="X8" s="10" t="s">
-        <x:v>47</x:v>
-      </x:c>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W8" s="10" t="s"/>
+      <x:c r="X8" s="10" t="s"/>
       <x:c r="Y8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Z8" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AA8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AB8" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AC8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AD8" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AE8" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="AF8" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="AG8" s="10" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="AH8" s="10" t="s"/>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH8" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AI8" s="10" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="AJ8" s="10" t="s"/>
+      <x:c r="AK8" s="10" t="s"/>
     </x:row>
     <x:row r="9" hidden="0">
       <x:c r="A9">
@@ -1501,100 +1553,210 @@
         <x:v>46091.8054166667</x:v>
       </x:c>
       <x:c r="D9" s="10" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E9" s="10" t="s"/>
       <x:c r="F9" s="2"/>
       <x:c r="G9" s="7" t="s">
-        <x:v>60</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H9" s="10" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I9" s="10" t="s">
-        <x:v>62</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="J9" s="10" t="s">
-        <x:v>51</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="K9" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M9" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P9" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q9" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="R9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="S9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T9" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="U9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="V9" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W9" s="10" t="s"/>
+      <x:c r="X9" s="10" t="s"/>
+      <x:c r="Y9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z9" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB9" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AC9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD9" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AE9" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF9" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AG9" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH9" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI9" s="10" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="AJ9" s="10" t="s"/>
+      <x:c r="AK9" s="10" t="s">
+        <x:v>67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" hidden="0">
+      <x:c r="A10">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B10" s="2">
+        <x:v>46093.458912037</x:v>
+      </x:c>
+      <x:c r="C10" s="2">
+        <x:v>46093.4646064815</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="s"/>
+      <x:c r="F10" s="2"/>
+      <x:c r="G10" s="7" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="H10" s="10" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="I10" s="10" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="L9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="M9" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="N9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="O9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="P9" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="Q9" s="10" t="s">
+      <x:c r="J10" s="10" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="R9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="S9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="T9" s="10" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="U9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="V9" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="W9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="X9" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="Y9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="Z9" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="AA9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="AB9" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="AC9" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="AD9" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="AE9" s="10" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="AF9" s="10" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="AG9" s="10" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="AH9" s="10" t="s">
-        <x:v>64</x:v>
-      </x:c>
+      <x:c r="K10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P10" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Q10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="T10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="U10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="X10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Y10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Z10" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB10" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AC10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AD10" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AE10" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF10" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AG10" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH10" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AI10" s="10" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="AJ10" s="10" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="AK10" s="10" t="s"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="Rccdafdd8c50d4c97"/>
+    <x:tablePart r:id="R556c54c27d094ec5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
More 8 user tests
</commit_message>
<xml_diff>
--- a/UserTests/Results/UserTestResultsWave2.xlsx
+++ b/UserTests/Results/UserTestResultsWave2.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <x:si>
     <x:t xml:space="preserve">ID</x:t>
   </x:si>
@@ -308,6 +308,60 @@
 Diminuir a distância entre as caixas de diálogos dos mini jogos  e o jogador ou aumentar estas caixas.
 Ter a possibilidade de customizar o avatar/mãos
 </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">O jogo do arco e flecha é bastante intuitivo e facil de jogar, ja o do frisbee ja nao era tao intuitivo na questao do reconhecimento dos movimentos do braço, de resto achei que foi tudoo bastante intuitivo e facil de compreender, aconcelho a alterar a fonte das instruçoes ou até dita-las em formato audio.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Acho que foi tudo relativamente bem ajustado, no jogo do arco e flecha a dificuldade foi aumentando, e o no frisbee as areas foram se ajustando a minha dificuldade.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Como ja tinha referido anteriormente apenas tive dificuldade a ler as instruções devido a fonte utilizada mas de resto nada apontar </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unemployed</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Gostei do ajuste automático à minha performance, apesar de pensar que poderia ser um pouco mais gradual esse ajuste. </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">uma única sugestão que teria seria maior diversidade de jogos.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">The main menu was kinda bugged, maybe I had the VR googles badly placed in my head but i had to look at strange places for the button and text of the mini-game to appear.
+What I liked the most was the bow and arrow game, very intuitive and was genuinely having fun. Played it 3 times and would play it 10 more.
+In the frisbee game I couldn't crack the mechanic but was still fun, but it didn't motivated me to play more</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">One fun thing I tried was to press the button with the frisbee and it would be a cool small feature. Other than the main menu bug I talked earlier, I didn't experience any other issues.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Para uma primeira experiência em imersão virtual achei muito confortável, o texto foi básico e o ambiente simples o suficiente para perceber o contexto do jogo. Os 2 jogos apresentados foram divertidos, sinto que no jogo do frisbee às vezes o lançamento tornava-se um bocado awkward pelo que só depois de alguns lançamentos é que consegui entender mais ou menos como eu conseguiria lançar para onde eu queria. No jogo do arco e flecha achei-o bem otimizado e muito simples e intuitivo de usar, facilmente torna-se divertido e a dificuldade crescente é notável em ambos os jogos. O único defeito que encontrei no jogo do arco e flecha foi que o texto no background não era o bastante visivel pelo que ás vezes quando era preciso atirar contra os balões vermelhos eu não percebia logo á primeira. </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">O meu texto anterior praticamente mete todos os comentários sobre a minha experiencia.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Só tornar o objetivo do jogo atual mais visivel ou percetivel</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As to what I liked the most, it was the games. The way they were structured, the movements and skills necessary and the difficulty level were fun and engaging. It is really fun to play the games, it feels engaging and immersive.
+On the not so good aspects, the text boxes could use some simplification. Some information provided does not really add to the experience and can be taken out, and other can be resumed. Also, the text boxes are not that well readable. My suggestion is to change the way the text is presented, and shorten its length to a minimum. The user does not really need to know the technical details of the game, just the bare minimums to get the game going. This way, by having a faster start to play, the game could be much more fun.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Already given above: main thing is to reduce text boxes in the beginning and change their aspect for an easier reading.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Achei o jogo super acessível e dinâmico. </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">senti uma ligeira dificuldade quando tinha de executar movimentos para a minha esquerda</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">I liked a lot the bow and arrow mini-game, I found it very pleasing and enjoyable to play. The frisbee mini-game was a little bit harder.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">personal trainner</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -404,8 +458,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK18" insertRow="1" totalsRowShown="0">
-  <x:autoFilter ref="A1:AK18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK26" insertRow="1" totalsRowShown="0">
+  <x:autoFilter ref="A1:AK26"/>
   <x:tableColumns count="37">
     <x:tableColumn id="1" uniqueName="1" name="ID" dataDxfId="0"/>
     <x:tableColumn id="2" uniqueName="2" name="Start time" dataDxfId="3"/>
@@ -2678,11 +2732,863 @@
         <x:v>90</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" hidden="0">
+      <x:c r="A19">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B19" s="2">
+        <x:v>46095.6580555556</x:v>
+      </x:c>
+      <x:c r="C19" s="2">
+        <x:v>46095.6776041667</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="s"/>
+      <x:c r="F19" s="2"/>
+      <x:c r="G19" s="7" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="H19" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I19" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J19" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N19" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R19" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="S19" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="T19" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="U19" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="V19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W19" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="X19" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Y19" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z19" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB19" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AC19" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AD19" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE19" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF19" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG19" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH19" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AI19" s="10" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="AJ19" s="10" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="AK19" s="10" t="s">
+        <x:v>93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" hidden="0">
+      <x:c r="A20">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B20" s="2">
+        <x:v>46095.677650463</x:v>
+      </x:c>
+      <x:c r="C20" s="2">
+        <x:v>46095.6904398148</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="s"/>
+      <x:c r="F20" s="2"/>
+      <x:c r="G20" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H20" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I20" s="10" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="J20" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M20" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O20" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P20" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Q20" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="R20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="T20" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="U20" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="V20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W20" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="X20" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Y20" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z20" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA20" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB20" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AD20" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF20" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AG20" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH20" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI20" s="10" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="AJ20" s="10" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="AK20" s="10" t="s"/>
+    </x:row>
+    <x:row r="21" hidden="0">
+      <x:c r="A21">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B21" s="2">
+        <x:v>46095.6944328704</x:v>
+      </x:c>
+      <x:c r="C21" s="2">
+        <x:v>46095.7052893518</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="s"/>
+      <x:c r="F21" s="2"/>
+      <x:c r="G21" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H21" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I21" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J21" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K21" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L21" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O21" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P21" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="R21" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="S21" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="T21" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="U21" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="W21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="X21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Y21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z21" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB21" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD21" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AE21" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF21" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG21" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH21" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI21" s="10" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="AJ21" s="10" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="AK21" s="10" t="s"/>
+    </x:row>
+    <x:row r="22" hidden="0">
+      <x:c r="A22">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B22" s="2">
+        <x:v>46095.7053125</x:v>
+      </x:c>
+      <x:c r="C22" s="2">
+        <x:v>46095.7132407407</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="s"/>
+      <x:c r="F22" s="2"/>
+      <x:c r="G22" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H22" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I22" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J22" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L22" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M22" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O22" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S22" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T22" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="U22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="X22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Y22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Z22" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB22" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AC22" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD22" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AE22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF22" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG22" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH22" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI22" s="10" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="AJ22" s="10" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AK22" s="10" t="s">
+        <x:v>101</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" hidden="0">
+      <x:c r="A23">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B23" s="2">
+        <x:v>46095.713275463</x:v>
+      </x:c>
+      <x:c r="C23" s="2">
+        <x:v>46095.7205787037</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="s"/>
+      <x:c r="F23" s="2"/>
+      <x:c r="G23" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H23" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I23" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J23" s="10" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="K23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L23" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N23" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O23" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="P23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R23" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="S23" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="U23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W23" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="X23" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Y23" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z23" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB23" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AC23" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD23" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF23" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AG23" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH23" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI23" s="10" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="AJ23" s="10" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="AK23" s="10" t="s"/>
+    </x:row>
+    <x:row r="24" hidden="0">
+      <x:c r="A24">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B24" s="2">
+        <x:v>46095.740625</x:v>
+      </x:c>
+      <x:c r="C24" s="2">
+        <x:v>46095.7438194444</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="s"/>
+      <x:c r="F24" s="2"/>
+      <x:c r="G24" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H24" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I24" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J24" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R24" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="S24" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="T24" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="U24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W24" s="10" t="s"/>
+      <x:c r="X24" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Y24" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z24" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA24" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB24" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AC24" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD24" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE24" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF24" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG24" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH24" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI24" s="10" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="AJ24" s="10" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="AK24" s="10" t="s"/>
+    </x:row>
+    <x:row r="25" hidden="0">
+      <x:c r="A25">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B25" s="2">
+        <x:v>46095.7496990741</x:v>
+      </x:c>
+      <x:c r="C25" s="2">
+        <x:v>46095.7532407407</x:v>
+      </x:c>
+      <x:c r="D25" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E25" s="10" t="s"/>
+      <x:c r="F25" s="2"/>
+      <x:c r="G25" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H25" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I25" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J25" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="L25" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="M25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Q25" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R25" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S25" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="T25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="U25" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V25" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="X25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Y25" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Z25" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB25" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD25" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AE25" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF25" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG25" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH25" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI25" s="10" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AJ25" s="10" t="s"/>
+      <x:c r="AK25" s="10" t="s"/>
+    </x:row>
+    <x:row r="26" hidden="0">
+      <x:c r="A26">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B26" s="2">
+        <x:v>46095.7572916667</x:v>
+      </x:c>
+      <x:c r="C26" s="2">
+        <x:v>46095.7599884259</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="s"/>
+      <x:c r="F26" s="2"/>
+      <x:c r="G26" s="7" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="H26" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I26" s="10" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="J26" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K26" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="L26" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S26" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T26" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="U26" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="V26" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="W26" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="X26" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Y26" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z26" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB26" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AC26" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD26" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF26" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AG26" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH26" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI26" s="10" t="s"/>
+      <x:c r="AJ26" s="10" t="s"/>
+      <x:c r="AK26" s="10" t="s"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R01aab36103f84c47"/>
+    <x:tablePart r:id="Re9e0cc50be4f4d46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Personalization Module Updated, results and notes for user tests (26 to 30)
</commit_message>
<xml_diff>
--- a/UserTests/Results/UserTestResultsWave2.xlsx
+++ b/UserTests/Results/UserTestResultsWave2.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
   <x:si>
     <x:t xml:space="preserve">ID</x:t>
   </x:si>
@@ -362,6 +362,15 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">personal trainner</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Gostei do arco e flecha, se pudesse controlar melhorar e ter maior range para controlar seria melhor. O frisbee as vezes não responde completamente como esperava, mas é divertido, eu meteria zonas laranjas mais longe também</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Para mim não é intuitivo ter de olhar para o jogo para que apareça o botão, penso que ficava muito longe e ficava numa posição estranha ao escolher o jogo</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">O ambiente e o jogo do arco e flecha</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -458,8 +467,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK26" insertRow="1" totalsRowShown="0">
-  <x:autoFilter ref="A1:AK26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK31" insertRow="1" totalsRowShown="0">
+  <x:autoFilter ref="A1:AK31"/>
   <x:tableColumns count="37">
     <x:tableColumn id="1" uniqueName="1" name="ID" dataDxfId="0"/>
     <x:tableColumn id="2" uniqueName="2" name="Start time" dataDxfId="3"/>
@@ -3584,11 +3593,530 @@
       <x:c r="AJ26" s="10" t="s"/>
       <x:c r="AK26" s="10" t="s"/>
     </x:row>
+    <x:row r="27" hidden="0">
+      <x:c r="A27">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B27" s="2">
+        <x:v>46099.4590972222</x:v>
+      </x:c>
+      <x:c r="C27" s="2">
+        <x:v>46099.4632407407</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E27" s="10" t="s"/>
+      <x:c r="F27" s="2"/>
+      <x:c r="G27" s="7" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="H27" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I27" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J27" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="R27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="U27" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="V27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="X27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Y27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z27" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB27" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD27" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AE27" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF27" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG27" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH27" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI27" s="10" t="s"/>
+      <x:c r="AJ27" s="10" t="s"/>
+      <x:c r="AK27" s="10" t="s"/>
+    </x:row>
+    <x:row r="28" hidden="0">
+      <x:c r="A28">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B28" s="2">
+        <x:v>46099.4659259259</x:v>
+      </x:c>
+      <x:c r="C28" s="2">
+        <x:v>46099.4738657407</x:v>
+      </x:c>
+      <x:c r="D28" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E28" s="10" t="s"/>
+      <x:c r="F28" s="2"/>
+      <x:c r="G28" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H28" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I28" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J28" s="10" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="K28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="L28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Q28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="R28" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="S28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T28" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="U28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="V28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="W28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="X28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Y28" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Z28" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AC28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD28" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF28" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG28" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH28" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AI28" s="10" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="AJ28" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="AK28" s="10" t="s">
+        <x:v>109</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" hidden="0">
+      <x:c r="A29">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B29" s="2">
+        <x:v>46099.4723958333</x:v>
+      </x:c>
+      <x:c r="C29" s="2">
+        <x:v>46099.477662037</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E29" s="10" t="s"/>
+      <x:c r="F29" s="2"/>
+      <x:c r="G29" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H29" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I29" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J29" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K29" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="L29" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M29" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="N29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S29" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="T29" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="U29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="X29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Y29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Z29" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA29" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB29" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AC29" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AD29" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE29" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF29" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG29" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH29" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI29" s="10" t="s"/>
+      <x:c r="AJ29" s="10" t="s"/>
+      <x:c r="AK29" s="10" t="s"/>
+    </x:row>
+    <x:row r="30" hidden="0">
+      <x:c r="A30">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B30" s="2">
+        <x:v>46099.4820138889</x:v>
+      </x:c>
+      <x:c r="C30" s="2">
+        <x:v>46099.4831944444</x:v>
+      </x:c>
+      <x:c r="D30" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E30" s="10" t="s"/>
+      <x:c r="F30" s="2"/>
+      <x:c r="G30" s="7" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="H30" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I30" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J30" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="T30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="U30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="X30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Y30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Z30" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB30" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AC30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AD30" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AE30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF30" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AG30" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH30" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI30" s="10" t="s"/>
+      <x:c r="AJ30" s="10" t="s"/>
+      <x:c r="AK30" s="10" t="s"/>
+    </x:row>
+    <x:row r="31" hidden="0">
+      <x:c r="A31">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B31" s="2">
+        <x:v>46099.4921643518</x:v>
+      </x:c>
+      <x:c r="C31" s="2">
+        <x:v>46099.4954513889</x:v>
+      </x:c>
+      <x:c r="D31" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="s"/>
+      <x:c r="F31" s="2"/>
+      <x:c r="G31" s="7" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="H31" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I31" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J31" s="10" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="K31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L31" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="O31" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Q31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S31" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="U31" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="V31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W31" s="10" t="s"/>
+      <x:c r="X31" s="10" t="s"/>
+      <x:c r="Y31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Z31" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB31" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AC31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AD31" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AE31" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF31" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG31" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH31" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI31" s="10" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="AJ31" s="10" t="s"/>
+      <x:c r="AK31" s="10" t="s"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="Re9e0cc50be4f4d46"/>
+    <x:tablePart r:id="Ra88e0aaefeb34a74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Results for User Tests from participant 33-35
</commit_message>
<xml_diff>
--- a/UserTests/Results/UserTestResultsWave2.xlsx
+++ b/UserTests/Results/UserTestResultsWave2.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
   <x:si>
     <x:t xml:space="preserve">ID</x:t>
   </x:si>
@@ -371,6 +371,27 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">O ambiente e o jogo do arco e flecha</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">O que gostei mais foi o conceito ser interessante </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Nop</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Os jogos em sí</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Adaptar para esquerdistas algumas circunstâncias do jogo </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">O conceito pareceu me interessante, tem só alguma complexidade onde as vezes posicionar as mãos </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">O sistema é intuitivo e fácil de usar, os jogos mantém se intressantes mesmo ao logo da sessão, e é interativo.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Alargar o número de mini-jogos para que exista mais variedade, e adicionar movimentação dentro do menu principal, de modo a que o jogador possa interagir melhor com o ambiente ao redor e ir de encontro às tendas para escolher o mini-game.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -467,8 +488,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK33" insertRow="1" totalsRowShown="0">
-  <x:autoFilter ref="A1:AK33"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK36" insertRow="1" totalsRowShown="0">
+  <x:autoFilter ref="A1:AK36"/>
   <x:tableColumns count="37">
     <x:tableColumn id="1" uniqueName="1" name="ID" dataDxfId="0"/>
     <x:tableColumn id="2" uniqueName="2" name="Start time" dataDxfId="3"/>
@@ -4318,11 +4339,334 @@
       <x:c r="AJ33" s="10" t="s"/>
       <x:c r="AK33" s="10" t="s"/>
     </x:row>
+    <x:row r="34" hidden="0">
+      <x:c r="A34">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B34" s="2">
+        <x:v>46100.981875</x:v>
+      </x:c>
+      <x:c r="C34" s="2">
+        <x:v>46100.9869097222</x:v>
+      </x:c>
+      <x:c r="D34" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E34" s="10" t="s"/>
+      <x:c r="F34" s="2"/>
+      <x:c r="G34" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H34" s="10" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="I34" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J34" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K34" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="L34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="P34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Q34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="R34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="S34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="T34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="U34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="V34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="W34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="X34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="Y34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Z34" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB34" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AC34" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD34" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AE34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AF34" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG34" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AH34" s="10" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AI34" s="10" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="AJ34" s="10" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="AK34" s="10" t="s"/>
+    </x:row>
+    <x:row r="35" hidden="0">
+      <x:c r="A35">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B35" s="2">
+        <x:v>46100.9818865741</x:v>
+      </x:c>
+      <x:c r="C35" s="2">
+        <x:v>46100.9877893518</x:v>
+      </x:c>
+      <x:c r="D35" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E35" s="10" t="s"/>
+      <x:c r="F35" s="2"/>
+      <x:c r="G35" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H35" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I35" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J35" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="L35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="O35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Q35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="R35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="S35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="U35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="V35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="W35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="X35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Y35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Z35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AA35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AB35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AC35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AE35" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AF35" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG35" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AH35" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AI35" s="10" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="AJ35" s="10" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="AK35" s="10" t="s">
+        <x:v>115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" hidden="0">
+      <x:c r="A36">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B36" s="2">
+        <x:v>46101.0207060185</x:v>
+      </x:c>
+      <x:c r="C36" s="2">
+        <x:v>46101.0315393518</x:v>
+      </x:c>
+      <x:c r="D36" s="10" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="s"/>
+      <x:c r="F36" s="2"/>
+      <x:c r="G36" s="7" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H36" s="10" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="I36" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J36" s="10" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="K36" s="10" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L36" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="M36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="P36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Q36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="R36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="S36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="T36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="U36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="V36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="W36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="X36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="Y36" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="Z36" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AA36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB36" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AC36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AD36" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AE36" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AF36" s="10" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AG36" s="10" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AH36" s="10" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AI36" s="10" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="AJ36" s="10" t="s"/>
+      <x:c r="AK36" s="10" t="s">
+        <x:v>117</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R4d2171fd61204772"/>
+    <x:tablePart r:id="R2cdf155f08cc4bf2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>